<commit_message>
update dashboard notifications and exams
</commit_message>
<xml_diff>
--- a/ai_model/attendance_log.xlsx
+++ b/ai_model/attendance_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,6 +519,60 @@
         </is>
       </c>
       <c r="E4" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>30409161402435</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mohamed Adel</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>12:40:07</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>23230035</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>zeyad wael</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>13:09:57</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>Present</t>
         </is>

</xml_diff>